<commit_message>
Pre Market Mon 2026-06-22
</commit_message>
<xml_diff>
--- a/market-prep/Pre Market 2026-06-22.xlsx
+++ b/market-prep/Pre Market 2026-06-22.xlsx
@@ -459,7 +459,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>7500,62</t>
+          <t>7500,57</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -476,7 +476,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>30447,85</t>
+          <t>30406,19</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -493,7 +493,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2979,70</t>
+          <t>2979,77</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -510,7 +510,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>51565,37</t>
+          <t>51564,71</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -595,7 +595,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>4215,31</t>
+          <t>4219,48</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -612,7 +612,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>65,78</t>
+          <t>65,65</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1697,29</t>
+          <t>1696,00</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>79,51</t>
+          <t>79,85</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>63125,99</t>
+          <t>62881,91</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -680,7 +680,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1711,80</t>
+          <t>1702,24</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -724,7 +724,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-10,52%</t>
+          <t>-11,06%</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -750,7 +750,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>7501,83</t>
+          <t>7500,58</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -768,7 +768,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>38</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>

</xml_diff>